<commit_message>
Added monte carlo sim
</commit_message>
<xml_diff>
--- a/clue_scroll.xlsx
+++ b/clue_scroll.xlsx
@@ -120,14 +120,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
-        <bgColor rgb="FF5EB91E"/>
+        <fgColor rgb="FF99CCFF"/>
+        <bgColor rgb="FFB3CAC7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF99CCFF"/>
-        <bgColor rgb="FFB3CAC7"/>
+        <fgColor rgb="FF00FF00"/>
+        <bgColor rgb="FF5EB91E"/>
       </patternFill>
     </fill>
     <fill>
@@ -218,10 +218,10 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -264,7 +264,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -273,7 +273,7 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -31534,13 +31534,13 @@
         </is>
       </c>
       <c r="D3" s="21" t="n">
-        <v>881424558.4000001</v>
+        <v>720317906.5</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t>"2026-07-04 18:14"</t>
+          <t>"2026-07-05 16:37"</t>
         </is>
       </c>
     </row>
@@ -31789,50 +31789,50 @@
         </is>
       </c>
       <c r="C18" s="28" t="n">
-        <v>1655</v>
+        <v>1650</v>
       </c>
       <c r="D18" s="28" t="n">
-        <v>72.81999999999999</v>
+        <v>73.05</v>
       </c>
       <c r="E18" s="28" t="n">
-        <v>49127</v>
+        <v>48880</v>
       </c>
       <c r="F18" s="28" t="n">
         <v>250000</v>
       </c>
       <c r="G18" s="28" t="n">
-        <v>413750000</v>
+        <v>412500000</v>
       </c>
       <c r="H18" s="28" t="n">
-        <v>185207645.5</v>
+        <v>306809906.5</v>
       </c>
       <c r="I18" s="29" t="inlineStr">
         <is>
-          <t>-228542354.50</t>
+          <t>-105690093.50</t>
         </is>
       </c>
       <c r="J18" s="29" t="inlineStr">
         <is>
-          <t>-123.4%</t>
+          <t>-34.4%</t>
         </is>
       </c>
       <c r="K18" s="28" t="n">
-        <v>316994</v>
+        <v>319371</v>
       </c>
       <c r="L18" s="28" t="n">
-        <v>524625070</v>
+        <v>526962150</v>
       </c>
       <c r="M18" s="28" t="n">
-        <v>372396445.58</v>
+        <v>219103218.05</v>
       </c>
       <c r="N18" s="29" t="inlineStr">
         <is>
-          <t>-152228624.42</t>
+          <t>-307858931.95</t>
         </is>
       </c>
       <c r="O18" s="29" t="inlineStr">
         <is>
-          <t>-40.9%</t>
+          <t>-140.5%</t>
         </is>
       </c>
     </row>
@@ -31843,50 +31843,50 @@
         </is>
       </c>
       <c r="C19" s="28" t="n">
-        <v>2944</v>
+        <v>2797</v>
       </c>
       <c r="D19" s="28" t="n">
-        <v>156.52</v>
+        <v>156.28</v>
       </c>
       <c r="E19" s="28" t="n">
-        <v>49127</v>
+        <v>48880</v>
       </c>
       <c r="F19" s="28" t="n">
         <v>125000</v>
       </c>
       <c r="G19" s="28" t="n">
-        <v>368000000</v>
+        <v>349625000</v>
       </c>
       <c r="H19" s="28" t="n">
-        <v>186567645.5</v>
+        <v>185882406.5</v>
       </c>
       <c r="I19" s="29" t="inlineStr">
         <is>
-          <t>-181432354.50</t>
+          <t>-163742593.50</t>
         </is>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
-          <t>-97.2%</t>
+          <t>-88.1%</t>
         </is>
       </c>
       <c r="K19" s="28" t="n">
         <v>159662</v>
       </c>
       <c r="L19" s="28" t="n">
-        <v>470044928</v>
+        <v>446574614</v>
       </c>
       <c r="M19" s="28" t="n">
-        <v>221567395.74</v>
+        <v>220725143.86</v>
       </c>
       <c r="N19" s="29" t="inlineStr">
         <is>
-          <t>-248477532.26</t>
+          <t>-225849470.14</t>
         </is>
       </c>
       <c r="O19" s="29" t="inlineStr">
         <is>
-          <t>-112.1%</t>
+          <t>-102.3%</t>
         </is>
       </c>
     </row>
@@ -31897,50 +31897,50 @@
         </is>
       </c>
       <c r="C20" s="28" t="n">
-        <v>3723</v>
+        <v>3716</v>
       </c>
       <c r="D20" s="28" t="n">
-        <v>224.09</v>
+        <v>224.87</v>
       </c>
       <c r="E20" s="28" t="n">
-        <v>49127</v>
+        <v>48880</v>
       </c>
       <c r="F20" s="28" t="n">
         <v>62500</v>
       </c>
       <c r="G20" s="28" t="n">
-        <v>232687500</v>
+        <v>232250000</v>
       </c>
       <c r="H20" s="28" t="n">
-        <v>181008270.5</v>
+        <v>119301781.5</v>
       </c>
       <c r="I20" s="29" t="inlineStr">
         <is>
-          <t>-51679229.50</t>
+          <t>-112948218.50</t>
         </is>
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>-28.6%</t>
+          <t>-94.7%</t>
         </is>
       </c>
       <c r="K20" s="28" t="n">
-        <v>80631</v>
+        <v>79808</v>
       </c>
       <c r="L20" s="28" t="n">
-        <v>300189213</v>
+        <v>296566528</v>
       </c>
       <c r="M20" s="28" t="n">
-        <v>138302342.29</v>
+        <v>213719591.46</v>
       </c>
       <c r="N20" s="29" t="inlineStr">
         <is>
-          <t>-161886870.71</t>
+          <t>-82846936.54</t>
         </is>
       </c>
       <c r="O20" s="29" t="inlineStr">
         <is>
-          <t>-117.1%</t>
+          <t>-38.8%</t>
         </is>
       </c>
     </row>
@@ -32069,54 +32069,54 @@
     <row r="28" ht="15" customHeight="1" s="17">
       <c r="B28" s="30" t="inlineStr">
         <is>
-          <t>EARTH (Best NBD)</t>
+          <t>EARTH (Best Naive)</t>
         </is>
       </c>
       <c r="C28" s="28" t="n">
-        <v>1603</v>
+        <v>1655</v>
       </c>
       <c r="D28" s="28" t="n">
-        <v>629.87</v>
+        <v>640.87</v>
       </c>
       <c r="E28" s="28" t="n">
-        <v>164595</v>
+        <v>165658</v>
       </c>
       <c r="F28" s="28" t="n">
         <v>150000</v>
       </c>
       <c r="G28" s="28" t="n">
-        <v>240450000</v>
+        <v>248250000</v>
       </c>
       <c r="H28" s="28" t="n">
-        <v>385558145.5</v>
+        <v>968567906.5</v>
       </c>
       <c r="I28" s="31" t="inlineStr">
         <is>
-          <t>145108145.50</t>
+          <t>720317906.50</t>
         </is>
       </c>
       <c r="J28" s="31" t="inlineStr">
         <is>
-          <t>37.6%</t>
+          <t>74.4%</t>
         </is>
       </c>
       <c r="K28" s="28" t="n">
-        <v>190170</v>
+        <v>193013</v>
       </c>
       <c r="L28" s="28" t="n">
-        <v>304842510</v>
+        <v>319436515</v>
       </c>
       <c r="M28" s="28" t="n">
-        <v>1186267068.4</v>
+        <v>475801869.81</v>
       </c>
       <c r="N28" s="32" t="inlineStr">
         <is>
-          <t>881424558.40</t>
+          <t>156365354.81</t>
         </is>
       </c>
       <c r="O28" s="32" t="inlineStr">
         <is>
-          <t>74.3%</t>
+          <t>32.9%</t>
         </is>
       </c>
     </row>
@@ -32127,104 +32127,104 @@
         </is>
       </c>
       <c r="C29" s="28" t="n">
-        <v>2290</v>
+        <v>2264</v>
       </c>
       <c r="D29" s="28" t="n">
-        <v>414.56</v>
+        <v>417.54</v>
       </c>
       <c r="E29" s="28" t="n">
-        <v>164595</v>
+        <v>165658</v>
       </c>
       <c r="F29" s="28" t="n">
         <v>75000</v>
       </c>
       <c r="G29" s="28" t="n">
-        <v>171750000</v>
+        <v>169800000</v>
       </c>
       <c r="H29" s="28" t="n">
-        <v>322169645.5</v>
+        <v>489607906.5</v>
       </c>
       <c r="I29" s="31" t="inlineStr">
         <is>
-          <t>150419645.50</t>
+          <t>319807906.50</t>
         </is>
       </c>
       <c r="J29" s="31" t="inlineStr">
         <is>
-          <t>46.7%</t>
+          <t>65.3%</t>
         </is>
       </c>
       <c r="K29" s="28" t="n">
-        <v>95779</v>
+        <v>96488</v>
       </c>
       <c r="L29" s="28" t="n">
-        <v>219333910</v>
+        <v>218448832</v>
       </c>
       <c r="M29" s="28" t="n">
-        <v>594464977.74</v>
+        <v>392393228.02</v>
       </c>
       <c r="N29" s="32" t="inlineStr">
         <is>
-          <t>375131067.74</t>
+          <t>173944396.02</t>
         </is>
       </c>
       <c r="O29" s="32" t="inlineStr">
         <is>
-          <t>63.1%</t>
+          <t>44.3%</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="17">
       <c r="B30" s="33" t="inlineStr">
         <is>
-          <t>ECLECTIC (Best Naive)</t>
+          <t>ECLECTIC (Best NBD)</t>
         </is>
       </c>
       <c r="C30" s="28" t="n">
-        <v>3953</v>
+        <v>3982</v>
       </c>
       <c r="D30" s="28" t="n">
-        <v>723.95</v>
+        <v>715.2</v>
       </c>
       <c r="E30" s="28" t="n">
-        <v>164595</v>
+        <v>165658</v>
       </c>
       <c r="F30" s="28" t="n">
         <v>37500</v>
       </c>
       <c r="G30" s="28" t="n">
-        <v>148237500</v>
+        <v>149325000</v>
       </c>
       <c r="H30" s="28" t="n">
-        <v>318225770.5</v>
+        <v>278039906.5</v>
       </c>
       <c r="I30" s="31" t="inlineStr">
         <is>
-          <t>169988270.50</t>
+          <t>128714906.50</t>
         </is>
       </c>
       <c r="J30" s="31" t="inlineStr">
         <is>
-          <t>53.4%</t>
+          <t>46.3%</t>
         </is>
       </c>
       <c r="K30" s="28" t="n">
-        <v>48365</v>
+        <v>48226</v>
       </c>
       <c r="L30" s="28" t="n">
-        <v>191186845</v>
+        <v>192035932</v>
       </c>
       <c r="M30" s="28" t="n">
-        <v>333992047.25</v>
+        <v>386596863.7</v>
       </c>
       <c r="N30" s="32" t="inlineStr">
         <is>
-          <t>142805202.25</t>
+          <t>194560931.70</t>
         </is>
       </c>
       <c r="O30" s="32" t="inlineStr">
         <is>
-          <t>42.8%</t>
+          <t>50.3%</t>
         </is>
       </c>
     </row>
@@ -32353,54 +32353,54 @@
     <row r="38" ht="15" customHeight="1" s="17">
       <c r="B38" s="30" t="inlineStr">
         <is>
-          <t>NATURE (Best NBD)</t>
+          <t>NATURE (Best Naive)</t>
         </is>
       </c>
       <c r="C38" s="28" t="n">
-        <v>4880</v>
+        <v>4882</v>
       </c>
       <c r="D38" s="28" t="n">
-        <v>1082.4</v>
+        <v>1077.36</v>
       </c>
       <c r="E38" s="28" t="n">
-        <v>186433.37</v>
+        <v>186348.29</v>
       </c>
       <c r="F38" s="28" t="n">
         <v>15000</v>
       </c>
       <c r="G38" s="28" t="n">
-        <v>73200000</v>
+        <v>73230000</v>
       </c>
       <c r="H38" s="28" t="n">
-        <v>53038034.6</v>
-      </c>
-      <c r="I38" s="29" t="inlineStr">
-        <is>
-          <t>-20161965.40</t>
-        </is>
-      </c>
-      <c r="J38" s="29" t="inlineStr">
-        <is>
-          <t>-38.0%</t>
+        <v>211338171.3</v>
+      </c>
+      <c r="I38" s="31" t="inlineStr">
+        <is>
+          <t>138108171.30</t>
+        </is>
+      </c>
+      <c r="J38" s="31" t="inlineStr">
+        <is>
+          <t>65.3%</t>
         </is>
       </c>
       <c r="K38" s="28" t="n">
-        <v>24472</v>
+        <v>25853</v>
       </c>
       <c r="L38" s="28" t="n">
-        <v>119423360</v>
+        <v>126214346</v>
       </c>
       <c r="M38" s="28" t="n">
-        <v>327653046.06</v>
-      </c>
-      <c r="N38" s="32" t="inlineStr">
-        <is>
-          <t>208229686.06</t>
-        </is>
-      </c>
-      <c r="O38" s="32" t="inlineStr">
-        <is>
-          <t>63.6%</t>
+        <v>80101620.95</v>
+      </c>
+      <c r="N38" s="29" t="inlineStr">
+        <is>
+          <t>-46112725.05</t>
+        </is>
+      </c>
+      <c r="O38" s="29" t="inlineStr">
+        <is>
+          <t>-57.6%</t>
         </is>
       </c>
     </row>
@@ -32411,50 +32411,50 @@
         </is>
       </c>
       <c r="C39" s="28" t="n">
-        <v>23029</v>
+        <v>23375</v>
       </c>
       <c r="D39" s="28" t="n">
-        <v>13165.15</v>
+        <v>13103.5</v>
       </c>
       <c r="E39" s="28" t="n">
-        <v>186433.37</v>
+        <v>186348.29</v>
       </c>
       <c r="F39" s="28" t="n">
         <v>7500</v>
       </c>
       <c r="G39" s="28" t="n">
-        <v>172717500</v>
+        <v>175312500</v>
       </c>
       <c r="H39" s="28" t="n">
-        <v>135540659.6</v>
-      </c>
-      <c r="I39" s="29" t="inlineStr">
-        <is>
-          <t>-37176840.40</t>
-        </is>
-      </c>
-      <c r="J39" s="29" t="inlineStr">
-        <is>
-          <t>-27.4%</t>
+        <v>200279876.3</v>
+      </c>
+      <c r="I39" s="31" t="inlineStr">
+        <is>
+          <t>24967376.30</t>
+        </is>
+      </c>
+      <c r="J39" s="31" t="inlineStr">
+        <is>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="K39" s="28" t="n">
-        <v>12405</v>
+        <v>12920</v>
       </c>
       <c r="L39" s="28" t="n">
-        <v>285674745</v>
+        <v>302005000</v>
       </c>
       <c r="M39" s="28" t="n">
-        <v>317941610.1900001</v>
-      </c>
-      <c r="N39" s="32" t="inlineStr">
-        <is>
-          <t>32266865.19</t>
-        </is>
-      </c>
-      <c r="O39" s="32" t="inlineStr">
-        <is>
-          <t>10.1%</t>
+        <v>221545852.87</v>
+      </c>
+      <c r="N39" s="29" t="inlineStr">
+        <is>
+          <t>-80459147.13</t>
+        </is>
+      </c>
+      <c r="O39" s="29" t="inlineStr">
+        <is>
+          <t>-36.3%</t>
         </is>
       </c>
     </row>
@@ -32465,50 +32465,50 @@
         </is>
       </c>
       <c r="C40" s="28" t="n">
-        <v>39734</v>
+        <v>40691</v>
       </c>
       <c r="D40" s="28" t="n">
-        <v>11979.84</v>
+        <v>11945.32</v>
       </c>
       <c r="E40" s="28" t="n">
-        <v>186433.37</v>
+        <v>186348.29</v>
       </c>
       <c r="F40" s="28" t="n">
         <v>3750</v>
       </c>
       <c r="G40" s="28" t="n">
-        <v>149002500</v>
+        <v>152591250</v>
       </c>
       <c r="H40" s="28" t="n">
-        <v>81726434.59999999</v>
+        <v>100211503.8</v>
       </c>
       <c r="I40" s="29" t="inlineStr">
         <is>
-          <t>-67276065.40</t>
+          <t>-52379746.20</t>
         </is>
       </c>
       <c r="J40" s="29" t="inlineStr">
         <is>
-          <t>-82.3%</t>
+          <t>-52.3%</t>
         </is>
       </c>
       <c r="K40" s="28" t="n">
-        <v>6329</v>
+        <v>6454</v>
       </c>
       <c r="L40" s="28" t="n">
-        <v>251476486</v>
+        <v>262619714</v>
       </c>
       <c r="M40" s="28" t="n">
-        <v>157366450.76</v>
+        <v>129343728.15</v>
       </c>
       <c r="N40" s="29" t="inlineStr">
         <is>
-          <t>-94110035.24</t>
+          <t>-133275985.85</t>
         </is>
       </c>
       <c r="O40" s="29" t="inlineStr">
         <is>
-          <t>-59.8%</t>
+          <t>-103.0%</t>
         </is>
       </c>
     </row>
@@ -32641,50 +32641,50 @@
         </is>
       </c>
       <c r="C48" s="28" t="n">
-        <v>454577</v>
+        <v>454601</v>
       </c>
       <c r="D48" s="28" t="n">
-        <v>148006.11</v>
+        <v>149098.16</v>
       </c>
       <c r="E48" s="28" t="n">
-        <v>411891.66</v>
+        <v>411528.48</v>
       </c>
       <c r="F48" s="28" t="n">
         <v>12500</v>
       </c>
       <c r="G48" s="28" t="n">
-        <v>5682212500</v>
+        <v>5682512500</v>
       </c>
       <c r="H48" s="28" t="n">
-        <v>1997234435.5</v>
+        <v>2936695606.5</v>
       </c>
       <c r="I48" s="29" t="inlineStr">
         <is>
-          <t>-3684978064.50</t>
+          <t>-2745816893.50</t>
         </is>
       </c>
       <c r="J48" s="29" t="inlineStr">
         <is>
-          <t>-184.5%</t>
+          <t>-93.5%</t>
         </is>
       </c>
       <c r="K48" s="28" t="n">
-        <v>15922</v>
+        <v>16647</v>
       </c>
       <c r="L48" s="28" t="n">
-        <v>7237774994</v>
+        <v>7567742847</v>
       </c>
       <c r="M48" s="28" t="n">
-        <v>3678426358.24</v>
+        <v>2651289133.94</v>
       </c>
       <c r="N48" s="29" t="inlineStr">
         <is>
-          <t>-3559348635.76</t>
+          <t>-4916453713.06</t>
         </is>
       </c>
       <c r="O48" s="29" t="inlineStr">
         <is>
-          <t>-96.8%</t>
+          <t>-185.4%</t>
         </is>
       </c>
     </row>

</xml_diff>